<commit_message>
fixed up analog channels
</commit_message>
<xml_diff>
--- a/git_cheat.xlsx
+++ b/git_cheat.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EtionData\ArduinoProjects\Ac1PhZC\Ac1PhZC3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E70C9270-8853-459E-93E2-C3C1683FC089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE1B390D-538F-44E4-BC6B-3F9AEE1C5ECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CF3A7945-7887-47A0-92C2-EFFFF36F6A90}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <r>
       <t xml:space="preserve"># Create new one pointing to new location
@@ -102,12 +102,84 @@
   <si>
     <t>show current branch</t>
   </si>
+  <si>
+    <t>git push --set-upstream origin ZCRetry</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">This links your local </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ZCRetry</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> branch to GitHub. After this first time, future pushes on this branch just need </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>git push</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>git</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> config --global push.autoSetupRemote </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF008080"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>true</t>
+    </r>
+  </si>
+  <si>
+    <t>To avoid this message for every new branch in future:</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -136,6 +208,18 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF008080"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -157,11 +241,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -189,10 +274,10 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>29049</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>2132169</xdr:colOff>
       <xdr:row>11</xdr:row>
-      <xdr:rowOff>129677</xdr:rowOff>
+      <xdr:rowOff>133487</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -525,19 +610,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E9CAF63-C308-445A-89D3-01021CEDC4CE}">
-  <dimension ref="B1:C13"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="B1:C15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="32.44140625" customWidth="1"/>
+    <col min="2" max="2" width="48.6640625" customWidth="1"/>
     <col min="3" max="3" width="46.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:3" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:3" ht="33.6" customHeight="1">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:3">
       <c r="B13" t="s">
         <v>1</v>
       </c>
@@ -545,6 +630,22 @@
         <v>2</v>
       </c>
     </row>
+    <row r="14" spans="2:3">
+      <c r="B14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3">
+      <c r="B15" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>